<commit_message>
feat: integrate saudi traffic violations calculator in ui and excel sheet
</commit_message>
<xml_diff>
--- a/نظام_تحليل_العملاء_الائتماني.xlsx
+++ b/نظام_تحليل_العملاء_الائتماني.xlsx
@@ -16,6 +16,8 @@
     <sheet name="6. الاعتمادات" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="7. أمر تنفيذ - تقرير" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="الإعدادات" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="8. حاسبة المخالفات" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="9. جدول المخالفات" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -29,7 +31,7 @@
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="30">
+  <fonts count="44">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -252,8 +254,83 @@
       <color rgb="FFFFFFFF"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <i val="1"/>
+      <color rgb="FF808080"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <color rgb="FF006100"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <color rgb="FF006100"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <color rgb="FF9C0006"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <i val="1"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="19">
+  <fills count="32">
     <fill>
       <patternFill/>
     </fill>
@@ -362,8 +439,73 @@
         <bgColor rgb="FFEBF5FB"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2E75B6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFACD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC00000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F7FC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFD699"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFBDD7EE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="19">
+  <borders count="24">
     <border>
       <left/>
       <right/>
@@ -595,6 +737,68 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thick">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thick">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thick">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFFFFFFF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFFFFFFF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFFFFFFF"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD3D3D3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD3D3D3"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD3D3D3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD3D3D3"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -606,7 +810,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="212">
+  <cellXfs count="244">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -1230,6 +1434,102 @@
     </xf>
     <xf numFmtId="0" fontId="29" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="19" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="20" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="21" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="22" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="19" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="23" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="23" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="19" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="19" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="19" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="19" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="24" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="25" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="25" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="20" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="19" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="26" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="26" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="26" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="27" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="28" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="28" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="28" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="29" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="30" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="31" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="25" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="20" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="20" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -4485,6 +4785,1029 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="0.7109375" customWidth="1" style="104" min="1" max="1"/>
+    <col width="38.28125" customWidth="1" style="104" min="2" max="2"/>
+    <col width="19.28125" customWidth="1" style="104" min="3" max="3"/>
+    <col width="15.00390625" customWidth="1" style="104" min="4" max="4"/>
+    <col width="19.28125" customWidth="1" style="104" min="5" max="5"/>
+    <col width="27.8515625" customWidth="1" style="104" min="6" max="6"/>
+    <col width="21.421875" customWidth="1" style="104" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1" s="104">
+      <c r="A1" s="212" t="inlineStr">
+        <is>
+          <t>حاسبة المخالفات المرورية - نظام المرور السعودي الجديد (10/04/2024)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16.5" customHeight="1" s="104">
+      <c r="A2" s="213" t="inlineStr">
+        <is>
+          <t>Saudi Traffic Violations Calculator - Effective 10/04/2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="21" customHeight="1" s="104">
+      <c r="A3" s="214" t="inlineStr">
+        <is>
+          <t>📌 ملاحظات مهمة</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="16.5" customHeight="1" s="104">
+      <c r="A4" s="215" t="inlineStr">
+        <is>
+          <t>• تخفيض 50% على المخالفات المرتكبة قبل تاريخ 18/04/2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="16.5" customHeight="1" s="104">
+      <c r="A5" s="215" t="inlineStr">
+        <is>
+          <t>• تخفيض 25% على المخالفات المرتكبة بعد 18/04/2024 (السداد خلال 30 يوماً)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16.5" customHeight="1" s="104">
+      <c r="A6" s="215" t="inlineStr">
+        <is>
+          <t>• مهلة الاعتراض 30 يوم | مهلة السداد 15 يوم | تمديد ممكن 90 يوم</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="16.5" customHeight="1" s="104">
+      <c r="A7" s="215" t="inlineStr">
+        <is>
+          <t>• بعد انتهاء المهلة: تطبق القيمة الكاملة بدون أي تخفيض</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
+    <row r="9" ht="33.75" customHeight="1" s="104">
+      <c r="B9" s="216" t="inlineStr">
+        <is>
+          <t>نوع المخالفة</t>
+        </is>
+      </c>
+      <c r="C9" s="216" t="inlineStr">
+        <is>
+          <t>قيمة الغرامة الأساسية (ريال)</t>
+        </is>
+      </c>
+      <c r="D9" s="216" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="E9" s="216" t="inlineStr">
+        <is>
+          <t>المجموع قبل الخصم</t>
+        </is>
+      </c>
+      <c r="F9" s="216" t="inlineStr">
+        <is>
+          <t>نوع التخفيض</t>
+        </is>
+      </c>
+      <c r="G9" s="216" t="inlineStr">
+        <is>
+          <t>المبلغ المستحق (ريال)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="19.5" customHeight="1" s="104">
+      <c r="B10" s="217" t="inlineStr">
+        <is>
+          <t>تجاوز الإشارة الحمراء</t>
+        </is>
+      </c>
+      <c r="C10" s="218" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D10" s="219" t="n"/>
+      <c r="E10" s="218">
+        <f>C10*D10</f>
+        <v/>
+      </c>
+      <c r="F10" s="220" t="inlineStr">
+        <is>
+          <t>بدون تخفيض</t>
+        </is>
+      </c>
+      <c r="G10" s="221">
+        <f>IF(F10="50% (قبل 18/04/2024)",E10*0.5,IF(F10="25% (بعد 18/04/2024)",E10*0.75,E10))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="19.5" customHeight="1" s="104">
+      <c r="B11" s="217" t="inlineStr">
+        <is>
+          <t>القيادة عكس الاتجاه</t>
+        </is>
+      </c>
+      <c r="C11" s="218" t="n">
+        <v>6000</v>
+      </c>
+      <c r="D11" s="219" t="n"/>
+      <c r="E11" s="218">
+        <f>C11*D11</f>
+        <v/>
+      </c>
+      <c r="F11" s="220" t="inlineStr">
+        <is>
+          <t>بدون تخفيض</t>
+        </is>
+      </c>
+      <c r="G11" s="221">
+        <f>IF(F11="50% (قبل 18/04/2024)",E11*0.5,IF(F11="25% (بعد 18/04/2024)",E11*0.75,E11))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="19.5" customHeight="1" s="104">
+      <c r="B12" s="217" t="inlineStr">
+        <is>
+          <t>تجاوز السرعة بأكثر من 25 كم/س</t>
+        </is>
+      </c>
+      <c r="C12" s="218" t="n">
+        <v>900</v>
+      </c>
+      <c r="D12" s="219" t="n"/>
+      <c r="E12" s="218">
+        <f>C12*D12</f>
+        <v/>
+      </c>
+      <c r="F12" s="220" t="inlineStr">
+        <is>
+          <t>بدون تخفيض</t>
+        </is>
+      </c>
+      <c r="G12" s="221">
+        <f>IF(F12="50% (قبل 18/04/2024)",E12*0.5,IF(F12="25% (بعد 18/04/2024)",E12*0.75,E12))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="19.5" customHeight="1" s="104">
+      <c r="B13" s="217" t="inlineStr">
+        <is>
+          <t>تجاوز السرعة بأقل من 25 كم/س</t>
+        </is>
+      </c>
+      <c r="C13" s="218" t="n">
+        <v>500</v>
+      </c>
+      <c r="D13" s="219" t="n"/>
+      <c r="E13" s="218">
+        <f>C13*D13</f>
+        <v/>
+      </c>
+      <c r="F13" s="220" t="inlineStr">
+        <is>
+          <t>بدون تخفيض</t>
+        </is>
+      </c>
+      <c r="G13" s="221">
+        <f>IF(F13="50% (قبل 18/04/2024)",E13*0.5,IF(F13="25% (بعد 18/04/2024)",E13*0.75,E13))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="19.5" customHeight="1" s="104">
+      <c r="B14" s="217" t="inlineStr">
+        <is>
+          <t>استخدام الجوال أثناء القيادة</t>
+        </is>
+      </c>
+      <c r="C14" s="218" t="n">
+        <v>500</v>
+      </c>
+      <c r="D14" s="219" t="n"/>
+      <c r="E14" s="218">
+        <f>C14*D14</f>
+        <v/>
+      </c>
+      <c r="F14" s="220" t="inlineStr">
+        <is>
+          <t>بدون تخفيض</t>
+        </is>
+      </c>
+      <c r="G14" s="221">
+        <f>IF(F14="50% (قبل 18/04/2024)",E14*0.5,IF(F14="25% (بعد 18/04/2024)",E14*0.75,E14))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="19.5" customHeight="1" s="104">
+      <c r="B15" s="217" t="inlineStr">
+        <is>
+          <t>عدم ربط حزام الأمان</t>
+        </is>
+      </c>
+      <c r="C15" s="218" t="n">
+        <v>150</v>
+      </c>
+      <c r="D15" s="219" t="n"/>
+      <c r="E15" s="218">
+        <f>C15*D15</f>
+        <v/>
+      </c>
+      <c r="F15" s="220" t="inlineStr">
+        <is>
+          <t>بدون تخفيض</t>
+        </is>
+      </c>
+      <c r="G15" s="221">
+        <f>IF(F15="50% (قبل 18/04/2024)",E15*0.5,IF(F15="25% (بعد 18/04/2024)",E15*0.75,E15))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="19.5" customHeight="1" s="104">
+      <c r="B16" s="217" t="inlineStr">
+        <is>
+          <t>القيادة بدون رخصة سارية</t>
+        </is>
+      </c>
+      <c r="C16" s="218" t="n">
+        <v>900</v>
+      </c>
+      <c r="D16" s="219" t="n"/>
+      <c r="E16" s="218">
+        <f>C16*D16</f>
+        <v/>
+      </c>
+      <c r="F16" s="220" t="inlineStr">
+        <is>
+          <t>بدون تخفيض</t>
+        </is>
+      </c>
+      <c r="G16" s="221">
+        <f>IF(F16="50% (قبل 18/04/2024)",E16*0.5,IF(F16="25% (بعد 18/04/2024)",E16*0.75,E16))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="19.5" customHeight="1" s="104">
+      <c r="B17" s="217" t="inlineStr">
+        <is>
+          <t>القيادة تحت تأثير المسكرات/المخدرات</t>
+        </is>
+      </c>
+      <c r="C17" s="218" t="n">
+        <v>9000</v>
+      </c>
+      <c r="D17" s="219" t="n"/>
+      <c r="E17" s="218">
+        <f>C17*D17</f>
+        <v/>
+      </c>
+      <c r="F17" s="220" t="inlineStr">
+        <is>
+          <t>بدون تخفيض</t>
+        </is>
+      </c>
+      <c r="G17" s="221">
+        <f>IF(F17="50% (قبل 18/04/2024)",E17*0.5,IF(F17="25% (بعد 18/04/2024)",E17*0.75,E17))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="19.5" customHeight="1" s="104">
+      <c r="B18" s="217" t="inlineStr">
+        <is>
+          <t>طمس لوحات المركبة</t>
+        </is>
+      </c>
+      <c r="C18" s="218" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D18" s="219" t="n"/>
+      <c r="E18" s="218">
+        <f>C18*D18</f>
+        <v/>
+      </c>
+      <c r="F18" s="220" t="inlineStr">
+        <is>
+          <t>بدون تخفيض</t>
+        </is>
+      </c>
+      <c r="G18" s="221">
+        <f>IF(F18="50% (قبل 18/04/2024)",E18*0.5,IF(F18="25% (بعد 18/04/2024)",E18*0.75,E18))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="19.5" customHeight="1" s="104">
+      <c r="B19" s="217" t="inlineStr">
+        <is>
+          <t>الوقوف في أماكن ذوي الإعاقة</t>
+        </is>
+      </c>
+      <c r="C19" s="218" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D19" s="219" t="n"/>
+      <c r="E19" s="218">
+        <f>C19*D19</f>
+        <v/>
+      </c>
+      <c r="F19" s="220" t="inlineStr">
+        <is>
+          <t>بدون تخفيض</t>
+        </is>
+      </c>
+      <c r="G19" s="221">
+        <f>IF(F19="50% (قبل 18/04/2024)",E19*0.5,IF(F19="25% (بعد 18/04/2024)",E19*0.75,E19))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="19.5" customHeight="1" s="104">
+      <c r="B20" s="217" t="inlineStr">
+        <is>
+          <t>عدم إعطاء أفضلية المرور للمشاة</t>
+        </is>
+      </c>
+      <c r="C20" s="218" t="n">
+        <v>500</v>
+      </c>
+      <c r="D20" s="219" t="n"/>
+      <c r="E20" s="218">
+        <f>C20*D20</f>
+        <v/>
+      </c>
+      <c r="F20" s="220" t="inlineStr">
+        <is>
+          <t>بدون تخفيض</t>
+        </is>
+      </c>
+      <c r="G20" s="221">
+        <f>IF(F20="50% (قبل 18/04/2024)",E20*0.5,IF(F20="25% (بعد 18/04/2024)",E20*0.75,E20))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="19.5" customHeight="1" s="104">
+      <c r="B21" s="217" t="inlineStr">
+        <is>
+          <t>تغيير المسار بشكل مفاجئ</t>
+        </is>
+      </c>
+      <c r="C21" s="218" t="n">
+        <v>300</v>
+      </c>
+      <c r="D21" s="219" t="n"/>
+      <c r="E21" s="218">
+        <f>C21*D21</f>
+        <v/>
+      </c>
+      <c r="F21" s="220" t="inlineStr">
+        <is>
+          <t>بدون تخفيض</t>
+        </is>
+      </c>
+      <c r="G21" s="221">
+        <f>IF(F21="50% (قبل 18/04/2024)",E21*0.5,IF(F21="25% (بعد 18/04/2024)",E21*0.75,E21))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="19.5" customHeight="1" s="104">
+      <c r="B22" s="217" t="inlineStr">
+        <is>
+          <t>عدم استخدام إشارات الانعطاف</t>
+        </is>
+      </c>
+      <c r="C22" s="218" t="n">
+        <v>150</v>
+      </c>
+      <c r="D22" s="219" t="n"/>
+      <c r="E22" s="218">
+        <f>C22*D22</f>
+        <v/>
+      </c>
+      <c r="F22" s="220" t="inlineStr">
+        <is>
+          <t>بدون تخفيض</t>
+        </is>
+      </c>
+      <c r="G22" s="221">
+        <f>IF(F22="50% (قبل 18/04/2024)",E22*0.5,IF(F22="25% (بعد 18/04/2024)",E22*0.75,E22))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="19.5" customHeight="1" s="104">
+      <c r="B23" s="217" t="inlineStr">
+        <is>
+          <t>تأخير تجديد رخصة القيادة</t>
+        </is>
+      </c>
+      <c r="C23" s="218" t="n">
+        <v>100</v>
+      </c>
+      <c r="D23" s="219" t="n"/>
+      <c r="E23" s="218">
+        <f>C23*D23</f>
+        <v/>
+      </c>
+      <c r="F23" s="220" t="inlineStr">
+        <is>
+          <t>بدون تخفيض</t>
+        </is>
+      </c>
+      <c r="G23" s="221">
+        <f>IF(F23="50% (قبل 18/04/2024)",E23*0.5,IF(F23="25% (بعد 18/04/2024)",E23*0.75,E23))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="19.5" customHeight="1" s="104">
+      <c r="B24" s="217" t="inlineStr">
+        <is>
+          <t>عدم تثبيت الحمولة أو تغطيتها</t>
+        </is>
+      </c>
+      <c r="C24" s="218" t="n">
+        <v>500</v>
+      </c>
+      <c r="D24" s="219" t="n"/>
+      <c r="E24" s="218">
+        <f>C24*D24</f>
+        <v/>
+      </c>
+      <c r="F24" s="220" t="inlineStr">
+        <is>
+          <t>بدون تخفيض</t>
+        </is>
+      </c>
+      <c r="G24" s="221">
+        <f>IF(F24="50% (قبل 18/04/2024)",E24*0.5,IF(F24="25% (بعد 18/04/2024)",E24*0.75,E24))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="28.5" customHeight="1" s="104">
+      <c r="B25" s="222" t="inlineStr">
+        <is>
+          <t>الإجمالي:</t>
+        </is>
+      </c>
+      <c r="C25" s="223" t="n"/>
+      <c r="D25" s="224">
+        <f>SUM(D10:D24)</f>
+        <v/>
+      </c>
+      <c r="E25" s="224">
+        <f>SUM(E10:E24)</f>
+        <v/>
+      </c>
+      <c r="F25" s="225" t="inlineStr">
+        <is>
+          <t>إجمالي المبلغ المستحق ←</t>
+        </is>
+      </c>
+      <c r="G25" s="226">
+        <f>SUM(G10:G24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="22.5" customHeight="1" s="104">
+      <c r="B26" s="227" t="inlineStr">
+        <is>
+          <t>💰 إجمالي المبلغ الموفر بفضل التخفيض:</t>
+        </is>
+      </c>
+      <c r="G26" s="228">
+        <f>E25-G25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27"/>
+    <row r="28" ht="19.5" customHeight="1" s="104">
+      <c r="A28" s="214" t="inlineStr">
+        <is>
+          <t>📝 طريقة الاستخدام:</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="16.5" customHeight="1" s="104">
+      <c r="A29" s="229" t="inlineStr">
+        <is>
+          <t>1️⃣ أدخل عدد المخالفات في عمود (العدد) - الخلايا الصفراء</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="16.5" customHeight="1" s="104">
+      <c r="A30" s="229" t="inlineStr">
+        <is>
+          <t>2️⃣ اختر نوع التخفيض من القائمة المنسدلة</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="16.5" customHeight="1" s="104">
+      <c r="A31" s="229" t="inlineStr">
+        <is>
+          <t>3️⃣ سيتم حساب المبلغ تلقائياً</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="16.5" customHeight="1" s="104">
+      <c r="A32" s="229" t="inlineStr">
+        <is>
+          <t>⚠️ المخالفات الجسيمة قد تشمل حجز المركبة + سجن</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="16.5" customHeight="1" s="104">
+      <c r="A33" s="229" t="inlineStr">
+        <is>
+          <t>📞 للاستعلام والسداد: منصة أبشر | تطبيق توكلني | 19911</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="0.7109375" customWidth="1" style="104" min="1" max="1"/>
+    <col width="1.140625" customWidth="1" style="104" min="2" max="2"/>
+    <col width="6.8515625" customWidth="1" style="104" min="3" max="3"/>
+    <col width="2.8515625" customWidth="1" style="104" min="4" max="4"/>
+    <col width="3.140625" customWidth="1" style="104" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="21" customHeight="1" s="104">
+      <c r="A1" s="212" t="inlineStr">
+        <is>
+          <t>جدول المخالفات المرورية الكامل - نظام المرور السعودي</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15.75" customHeight="1" s="104">
+      <c r="B2" s="230" t="inlineStr">
+        <is>
+          <t>الرقم</t>
+        </is>
+      </c>
+      <c r="C2" s="230" t="inlineStr">
+        <is>
+          <t>نوع المخالفة</t>
+        </is>
+      </c>
+      <c r="D2" s="230" t="inlineStr">
+        <is>
+          <t>قيمة الغرامة (ريال)</t>
+        </is>
+      </c>
+      <c r="E2" s="230" t="inlineStr">
+        <is>
+          <t>الفئة</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="19.5" customHeight="1" s="104">
+      <c r="B3" s="231" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="232" t="inlineStr">
+        <is>
+          <t>القيادة تحت تأثير المسكرات أو المخدرات</t>
+        </is>
+      </c>
+      <c r="D3" s="233" t="n">
+        <v>9000</v>
+      </c>
+      <c r="E3" s="234" t="inlineStr">
+        <is>
+          <t>جسيمة جداً</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="19.5" customHeight="1" s="104">
+      <c r="B4" s="235" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" s="236" t="inlineStr">
+        <is>
+          <t>القيادة عكس الاتجاه على الطرق السريعة</t>
+        </is>
+      </c>
+      <c r="D4" s="237" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E4" s="234" t="inlineStr">
+        <is>
+          <t>جسيمة جداً</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="19.5" customHeight="1" s="104">
+      <c r="B5" s="231" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" s="232" t="inlineStr">
+        <is>
+          <t>تركيب لوحات مزورة على المركبة</t>
+        </is>
+      </c>
+      <c r="D5" s="233" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E5" s="234" t="inlineStr">
+        <is>
+          <t>جسيمة جداً</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="19.5" customHeight="1" s="104">
+      <c r="B6" s="235" t="n">
+        <v>4</v>
+      </c>
+      <c r="C6" s="236" t="inlineStr">
+        <is>
+          <t>القيادة بتهور أو تفحيط</t>
+        </is>
+      </c>
+      <c r="D6" s="237" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E6" s="234" t="inlineStr">
+        <is>
+          <t>جسيمة جداً</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="19.5" customHeight="1" s="104">
+      <c r="B7" s="231" t="n">
+        <v>5</v>
+      </c>
+      <c r="C7" s="232" t="inlineStr">
+        <is>
+          <t>تجاوز الإشارة الحمراء</t>
+        </is>
+      </c>
+      <c r="D7" s="233" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E7" s="238" t="inlineStr">
+        <is>
+          <t>جسيمة</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="19.5" customHeight="1" s="104">
+      <c r="B8" s="235" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" s="236" t="inlineStr">
+        <is>
+          <t>طمس لوحات المركبة أو عدم حملها</t>
+        </is>
+      </c>
+      <c r="D8" s="237" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E8" s="238" t="inlineStr">
+        <is>
+          <t>جسيمة</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="19.5" customHeight="1" s="104">
+      <c r="B9" s="231" t="n">
+        <v>7</v>
+      </c>
+      <c r="C9" s="232" t="inlineStr">
+        <is>
+          <t>تغيير ملامح المركبة</t>
+        </is>
+      </c>
+      <c r="D9" s="233" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E9" s="239" t="inlineStr">
+        <is>
+          <t>خطيرة</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="19.5" customHeight="1" s="104">
+      <c r="B10" s="235" t="n">
+        <v>8</v>
+      </c>
+      <c r="C10" s="236" t="inlineStr">
+        <is>
+          <t>الوقوف في أماكن ذوي الإعاقة</t>
+        </is>
+      </c>
+      <c r="D10" s="237" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E10" s="239" t="inlineStr">
+        <is>
+          <t>خطيرة</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="19.5" customHeight="1" s="104">
+      <c r="B11" s="231" t="n">
+        <v>9</v>
+      </c>
+      <c r="C11" s="232" t="inlineStr">
+        <is>
+          <t>تجاوز السرعة بأكثر من 25 كم/س</t>
+        </is>
+      </c>
+      <c r="D11" s="233" t="n">
+        <v>900</v>
+      </c>
+      <c r="E11" s="239" t="inlineStr">
+        <is>
+          <t>خطيرة</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="19.5" customHeight="1" s="104">
+      <c r="B12" s="235" t="n">
+        <v>10</v>
+      </c>
+      <c r="C12" s="236" t="inlineStr">
+        <is>
+          <t>القيادة بدون رخصة قيادة سارية</t>
+        </is>
+      </c>
+      <c r="D12" s="237" t="n">
+        <v>900</v>
+      </c>
+      <c r="E12" s="239" t="inlineStr">
+        <is>
+          <t>خطيرة</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="19.5" customHeight="1" s="104">
+      <c r="B13" s="231" t="n">
+        <v>11</v>
+      </c>
+      <c r="C13" s="232" t="inlineStr">
+        <is>
+          <t>تجاوز السرعة بأقل من 25 كم/س</t>
+        </is>
+      </c>
+      <c r="D13" s="233" t="n">
+        <v>500</v>
+      </c>
+      <c r="E13" s="240" t="inlineStr">
+        <is>
+          <t>متوسطة</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="19.5" customHeight="1" s="104">
+      <c r="B14" s="235" t="n">
+        <v>12</v>
+      </c>
+      <c r="C14" s="236" t="inlineStr">
+        <is>
+          <t>استخدام الجوال أثناء القيادة</t>
+        </is>
+      </c>
+      <c r="D14" s="237" t="n">
+        <v>500</v>
+      </c>
+      <c r="E14" s="240" t="inlineStr">
+        <is>
+          <t>متوسطة</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="19.5" customHeight="1" s="104">
+      <c r="B15" s="231" t="n">
+        <v>13</v>
+      </c>
+      <c r="C15" s="232" t="inlineStr">
+        <is>
+          <t>عدم إعطاء أفضلية المرور للمشاة</t>
+        </is>
+      </c>
+      <c r="D15" s="233" t="n">
+        <v>500</v>
+      </c>
+      <c r="E15" s="240" t="inlineStr">
+        <is>
+          <t>متوسطة</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="19.5" customHeight="1" s="104">
+      <c r="B16" s="235" t="n">
+        <v>14</v>
+      </c>
+      <c r="C16" s="236" t="inlineStr">
+        <is>
+          <t>عدم تثبيت الحمولة أو تغطيتها</t>
+        </is>
+      </c>
+      <c r="D16" s="237" t="n">
+        <v>500</v>
+      </c>
+      <c r="E16" s="240" t="inlineStr">
+        <is>
+          <t>متوسطة</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="19.5" customHeight="1" s="104">
+      <c r="B17" s="231" t="n">
+        <v>15</v>
+      </c>
+      <c r="C17" s="232" t="inlineStr">
+        <is>
+          <t>تغيير المسار بشكل مفاجئ</t>
+        </is>
+      </c>
+      <c r="D17" s="233" t="n">
+        <v>300</v>
+      </c>
+      <c r="E17" s="240" t="inlineStr">
+        <is>
+          <t>متوسطة</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="19.5" customHeight="1" s="104">
+      <c r="B18" s="235" t="n">
+        <v>16</v>
+      </c>
+      <c r="C18" s="236" t="inlineStr">
+        <is>
+          <t>الوقوف على الرصيف</t>
+        </is>
+      </c>
+      <c r="D18" s="237" t="n">
+        <v>300</v>
+      </c>
+      <c r="E18" s="240" t="inlineStr">
+        <is>
+          <t>متوسطة</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="19.5" customHeight="1" s="104">
+      <c r="B19" s="231" t="n">
+        <v>17</v>
+      </c>
+      <c r="C19" s="232" t="inlineStr">
+        <is>
+          <t>عدم الالتزام بأنظمة الانتظار</t>
+        </is>
+      </c>
+      <c r="D19" s="233" t="n">
+        <v>300</v>
+      </c>
+      <c r="E19" s="240" t="inlineStr">
+        <is>
+          <t>متوسطة</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="19.5" customHeight="1" s="104">
+      <c r="B20" s="235" t="n">
+        <v>18</v>
+      </c>
+      <c r="C20" s="236" t="inlineStr">
+        <is>
+          <t>عدم ربط حزام الأمان</t>
+        </is>
+      </c>
+      <c r="D20" s="237" t="n">
+        <v>150</v>
+      </c>
+      <c r="E20" s="241" t="inlineStr">
+        <is>
+          <t>بسيطة</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="19.5" customHeight="1" s="104">
+      <c r="B21" s="231" t="n">
+        <v>19</v>
+      </c>
+      <c r="C21" s="232" t="inlineStr">
+        <is>
+          <t>عدم استخدام إشارات الانعطاف</t>
+        </is>
+      </c>
+      <c r="D21" s="233" t="n">
+        <v>150</v>
+      </c>
+      <c r="E21" s="241" t="inlineStr">
+        <is>
+          <t>بسيطة</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="19.5" customHeight="1" s="104">
+      <c r="B22" s="235" t="n">
+        <v>20</v>
+      </c>
+      <c r="C22" s="236" t="inlineStr">
+        <is>
+          <t>عدم وضع كرسي الأطفال للأقل من 8 سنوات</t>
+        </is>
+      </c>
+      <c r="D22" s="237" t="n">
+        <v>150</v>
+      </c>
+      <c r="E22" s="241" t="inlineStr">
+        <is>
+          <t>بسيطة</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="19.5" customHeight="1" s="104">
+      <c r="B23" s="231" t="n">
+        <v>21</v>
+      </c>
+      <c r="C23" s="232" t="inlineStr">
+        <is>
+          <t>تأخير تجديد رخصة القيادة</t>
+        </is>
+      </c>
+      <c r="D23" s="233" t="n">
+        <v>100</v>
+      </c>
+      <c r="E23" s="241" t="inlineStr">
+        <is>
+          <t>بسيطة</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="19.5" customHeight="1" s="104">
+      <c r="B24" s="235" t="n">
+        <v>22</v>
+      </c>
+      <c r="C24" s="236" t="inlineStr">
+        <is>
+          <t>تأخير تجديد رخصة السير (الاستمارة)</t>
+        </is>
+      </c>
+      <c r="D24" s="237" t="n">
+        <v>100</v>
+      </c>
+      <c r="E24" s="241" t="inlineStr">
+        <is>
+          <t>بسيطة</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="19.5" customHeight="1" s="104">
+      <c r="B25" s="231" t="n">
+        <v>23</v>
+      </c>
+      <c r="C25" s="232" t="inlineStr">
+        <is>
+          <t>عدم حمل الرخصة أثناء القيادة</t>
+        </is>
+      </c>
+      <c r="D25" s="233" t="n">
+        <v>100</v>
+      </c>
+      <c r="E25" s="241" t="inlineStr">
+        <is>
+          <t>بسيطة</t>
+        </is>
+      </c>
+    </row>
+    <row r="26"/>
+    <row r="27" ht="18.75" customHeight="1" s="104">
+      <c r="B27" s="242" t="inlineStr">
+        <is>
+          <t>📌 المصدر: نظام المرور السعودي - الإدارة العامة للمرور | وزارة الداخلية www.moi.gov.sa</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="16.5" customHeight="1" s="104">
+      <c r="B28" s="243" t="inlineStr">
+        <is>
+          <t>نظام المرور الجديد - ساري المفعول من 10/04/2024 | جميع القيم بالريال السعودي</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">

</xml_diff>